<commit_message>
Melhora layout principal e valida prazo dos jogos
</commit_message>
<xml_diff>
--- a/jogos_loteria_nior.xlsx
+++ b/jogos_loteria_nior.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -462,7 +462,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>gs</t>
+          <t>Gustavo Mayan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -472,7 +472,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2 - 5 - 6 - 8 - 9 - 11 - 12 - 13 - 14 - 16 - 17 - 19 - 22 - 24 - 25</t>
+          <t>1 - 2 - 3 - 4 - 5 - 6 - 7 - 8 - 9 - 10 - 11 - 12 - 13 - 14 - 15</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -480,35 +480,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>08/09/2026 16:45:39</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>gs</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>gustavomayan113@gmail.com</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1 - 2 - 3 - 6 - 7 - 9 - 10 - 11 - 13 - 15 - 17 - 19 - 21 - 23 - 24</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>15</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>08/09/2026 16:47:22</t>
+          <t>09/09/2026 12:51:50</t>
         </is>
       </c>
     </row>

</xml_diff>